<commit_message>
Add the Neuvillette <-> NeuvilletteMelusent remap, compiled both ways
Mod types, hashes, indices, vertex counts and vertex-group rows for Neuvillette (4.0 / 4.3) and
NeuvilletteMelusent (6.3: an unnamed main mesh, Coat, Bang, Eye), a component-template fix with
four rows forward and a merge-template fix back, and both parsers. Transcribed from the two
prototypes, which stay the oracles: the compiled rows are byte-identical to them on ten forward
mods and six reverse ones (the identity, the one real skin mod and four synthetic ones built by
neuvilletteMelusentSynth.py).

The vertex-group rows carry the moves seen in game: his coat tails whole in the Coat, the skin's
mantle sleeves on his upper arms (and its right shoulder on the mirror of its left's bone), the
skin's cuff band on his forearms. The draft workbook agrees with every compiled row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
+++ b/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
@@ -459,7 +459,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -1077,15 +1076,15 @@
       <c r="A34" t="n">
         <v>32</v>
       </c>
-      <c r="B34" t="n">
-        <v>85</v>
+      <c r="D34" t="n">
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>0.44</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>204 verts (Body) -&gt; 178 verts (Head), dist 0.0507; runner-up 87 at dist 0.1077</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 204 verts (Body) -&gt; 178 verts (Head), dist 0.0507; runner-up 87 at dist 0.1077)</t>
         </is>
       </c>
     </row>
@@ -1093,15 +1092,15 @@
       <c r="A35" t="n">
         <v>33</v>
       </c>
-      <c r="B35" t="n">
-        <v>87</v>
+      <c r="D35" t="n">
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>0.964</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>702 verts (Body) -&gt; 173 verts (Head), dist 0.2631; runner-up 23 at dist 0.2112</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2631; runner-up 23 at dist 0.2112)</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1116,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 23 at dist 0.2687</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 23 at dist 0.2687)</t>
         </is>
       </c>
     </row>
@@ -1125,15 +1124,15 @@
       <c r="A37" t="n">
         <v>35</v>
       </c>
-      <c r="B37" t="n">
-        <v>85</v>
+      <c r="D37" t="n">
+        <v>7</v>
       </c>
       <c r="F37" t="n">
         <v>0.494</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>155 verts (Body) -&gt; 178 verts (Head), dist 0.1055; runner-up 70 at dist 0.1273</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 155 verts (Body) -&gt; 178 verts (Head), dist 0.1055; runner-up 70 at dist 0.1273)</t>
         </is>
       </c>
     </row>
@@ -1141,15 +1140,15 @@
       <c r="A38" t="n">
         <v>36</v>
       </c>
-      <c r="B38" t="n">
-        <v>87</v>
+      <c r="D38" t="n">
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>0.667</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>209 verts (Body) -&gt; 173 verts (Head), dist 0.1485; runner-up Coat:7 at dist 0.1508</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 209 verts (Body) -&gt; 173 verts (Head), dist 0.1485; runner-up Coat:7 at dist 0.1508)</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1164,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:9 at dist 0.2280</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:9 at dist 0.2280)</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1180,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:21 at dist 0.3067</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:21 at dist 0.3067)</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1196,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Reviewed: tip of the long back coat tail (cyan trim); the skin coat's tail end, not the skin's CALF (cloth onto a leg). Tool proposed 6. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:24 at dist 0.3440)</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail (cyan trim); the skin coat's tail end, not the skin's CALF (cloth onto a leg). Tool proposed 6. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:24 at dist 0.3440))</t>
         </is>
       </c>
     </row>
@@ -1205,15 +1204,15 @@
       <c r="A42" t="n">
         <v>40</v>
       </c>
-      <c r="B42" t="n">
-        <v>86</v>
+      <c r="D42" t="n">
+        <v>8</v>
       </c>
       <c r="F42" t="n">
         <v>0.439</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>204 verts (Body) -&gt; 178 verts (Head), dist 0.0507; runner-up 88 at dist 0.1077</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 204 verts (Body) -&gt; 178 verts (Head), dist 0.0507; runner-up 88 at dist 0.1077)</t>
         </is>
       </c>
     </row>
@@ -1221,15 +1220,15 @@
       <c r="A43" t="n">
         <v>41</v>
       </c>
-      <c r="B43" t="n">
-        <v>88</v>
+      <c r="D43" t="n">
+        <v>10</v>
       </c>
       <c r="F43" t="n">
         <v>0.962</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>702 verts (Body) -&gt; 173 verts (Head), dist 0.2630; runner-up 43 at dist 0.2113</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2630; runner-up 43 at dist 0.2113)</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1244,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 43 at dist 0.2687</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 43 at dist 0.2687)</t>
         </is>
       </c>
     </row>
@@ -1253,15 +1252,15 @@
       <c r="A45" t="n">
         <v>43</v>
       </c>
-      <c r="B45" t="n">
-        <v>86</v>
+      <c r="D45" t="n">
+        <v>8</v>
       </c>
       <c r="F45" t="n">
         <v>0.405</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>155 verts (Body) -&gt; 178 verts (Head), dist 0.1055; runner-up 71 at dist 0.1310</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 155 verts (Body) -&gt; 178 verts (Head), dist 0.1055; runner-up 71 at dist 0.1310)</t>
         </is>
       </c>
     </row>
@@ -1269,15 +1268,15 @@
       <c r="A46" t="n">
         <v>44</v>
       </c>
-      <c r="B46" t="n">
-        <v>88</v>
+      <c r="D46" t="n">
+        <v>10</v>
       </c>
       <c r="F46" t="n">
         <v>0.576</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>209 verts (Body) -&gt; 173 verts (Head), dist 0.1485; runner-up Coat:8 at dist 0.1616</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 209 verts (Body) -&gt; 173 verts (Head), dist 0.1485; runner-up Coat:8 at dist 0.1616)</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1292,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:10 at dist 0.2280</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:10 at dist 0.2280)</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1308,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:22 at dist 0.3067</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:22 at dist 0.3067)</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1324,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Reviewed: tip of the long back coat tail, right; the skin coat's tail end, not the calf. Tool proposed 26. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:25 at dist 0.3440)</t>
+          <t>Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail, right; the skin coat's tail end, not the calf. Tool proposed 26. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:25 at dist 0.3440))</t>
         </is>
       </c>
     </row>
@@ -3324,14 +3323,14 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="C55" t="n">
         <v>0.872</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Reviewed: the skin's left sleeve cuff (forward 58 -&gt; 53); Neuvillette's cuff bone rather than a THUMB bone (111). Tool proposed 111. (220 verts (Head) -&gt; 103 verts (Body/Dress), dist 0.1007; runner-up 112 at dist 0.1332)</t>
+          <t>Reviewed (in game, 2026-09-25): the main mesh's cuff band onto his FOREARM (85 / 104, the bone his hand chain shares vertices with), not his separate cuff piece (58 / 61). (was: Reviewed: the skin's left sleeve cuff (forward 58 -&gt; 53); Neuvillette's cuff bone rather than a THUMB bone (111). Tool proposed 111. (220 verts (Head) -&gt; 103 verts (Body/Dress), dist 0.1007; runner-up 112 at dist 0.1332))</t>
         </is>
       </c>
     </row>
@@ -3340,14 +3339,14 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="C56" t="n">
         <v>0.698</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Reviewed: the skin's right sleeve cuff; Neuvillette's cuff bone rather than a thumb bone (113). Tool proposed 113. (218 verts (Head) -&gt; 155 verts (Body/Dress), dist 0.0733; runner-up 104 at dist 0.0706)</t>
+          <t>Reviewed (in game, 2026-09-25): the main mesh's cuff band onto his FOREARM (85 / 104, the bone his hand chain shares vertices with), not his separate cuff piece (58 / 61). (was: Reviewed: the skin's right sleeve cuff; Neuvillette's cuff bone rather than a thumb bone (113). Tool proposed 113. (218 verts (Head) -&gt; 155 verts (Body/Dress), dist 0.0733; runner-up 104 at dist 0.0706))</t>
         </is>
       </c>
     </row>
@@ -4438,14 +4437,14 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C16" t="n">
         <v>0.37</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>366 verts (A) -&gt; 163 verts (Body), dist 0.0650; runner-up 66 at dist 0.1276; in chain Coat:13-14 -&gt; 64-65</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the mantle's RIGHT shoulder onto 67, the mirror of its left twin's 64 (the draft had 65). (was: 366 verts (A) -&gt; 163 verts (Body), dist 0.0650; runner-up 66 at dist 0.1276; in chain Coat:13-14 -&gt; 64-65)</t>
         </is>
       </c>
     </row>
@@ -4710,14 +4709,14 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C33" t="n">
         <v>0.483</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>231 verts (A) -&gt; 163 verts (Body), dist 0.1051; runner-up 19 at dist 0.1795; in chain Coat:30-31 -&gt; 64-65</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the mantle's RIGHT shoulder onto 67, the mirror of its left twin's 64 (the draft had 65). (was: 231 verts (A) -&gt; 163 verts (Body), dist 0.1051; runner-up 19 at dist 0.1795; in chain Coat:30-31 -&gt; 64-65)</t>
         </is>
       </c>
     </row>
@@ -4726,14 +4725,14 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C34" t="n">
         <v>0.766</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Reviewed: coat's left UPPER SLEEVE (it runs down the arm in the front view); Neuvillette's upper-sleeve bone, not HAIR (20) -- cloth riding hair wobbles. Tool proposed 20. (308 verts (A) -&gt; 175 verts (Head), dist 0.0888; runner-up 57 at dist 0.1112)</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: Reviewed: coat's left UPPER SLEEVE (it runs down the arm in the front view); Neuvillette's upper-sleeve bone, not HAIR (20) -- cloth riding hair wobbles. Tool proposed 20. (308 verts (A) -&gt; 175 verts (Head), dist 0.0888; runner-up 57 at dist 0.1112))</t>
         </is>
       </c>
     </row>
@@ -4742,14 +4741,14 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C35" t="n">
         <v>0.727</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Reviewed: coat's right upper sleeve; Neuvillette's upper-sleeve bone, not HAIR (19). Tool proposed 19. (308 verts (A) -&gt; 175 verts (Head), dist 0.0888; runner-up 60 at dist 0.1112; in chain Coat:33-34 -&gt; 19-20)</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: Reviewed: coat's right upper sleeve; Neuvillette's upper-sleeve bone, not HAIR (19). Tool proposed 19. (308 verts (A) -&gt; 175 verts (Head), dist 0.0888; runner-up 60 at dist 0.1112; in chain Coat:33-34 -&gt; 19-20))</t>
         </is>
       </c>
     </row>
@@ -4758,14 +4757,14 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C36" t="n">
         <v>0.949</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Reviewed: coat sleeve, left, hanging behind the arm; Neuvillette's sleeve cuff (vertices mode), not HAIR (20). Tool proposed 20. (1452 verts (A) -&gt; 175 verts (Head), dist 0.2955; runner-up 58 at dist 0.2158; in chain Coat:33-34 -&gt; 19-20)</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: Reviewed: coat sleeve, left, hanging behind the arm; Neuvillette's sleeve cuff (vertices mode), not HAIR (20). Tool proposed 20. (1452 verts (A) -&gt; 175 verts (Head), dist 0.2955; runner-up 58 at dist 0.2158; in chain Coat:33-34 -&gt; 19-20))</t>
         </is>
       </c>
     </row>
@@ -4774,14 +4773,14 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C37" t="n">
         <v>0.621</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1452 verts (A) -&gt; 733 verts (Body), dist 0.2158; runner-up 99 at dist 0.2560</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: 1452 verts (A) -&gt; 733 verts (Body), dist 0.2158; runner-up 99 at dist 0.2560)</t>
         </is>
       </c>
     </row>
@@ -4790,14 +4789,14 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C38" t="n">
         <v>0.9340000000000001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Reviewed: coat sleeve, left, lower; the sleeve cuff (vertices mode), not a FINGER bone (82). Tool proposed 82. (1639 verts (A) -&gt; 53 verts (Body), dist 0.2577; runner-up 81 at dist 0.2635)</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: Reviewed: coat sleeve, left, lower; the sleeve cuff (vertices mode), not a FINGER bone (82). Tool proposed 82. (1639 verts (A) -&gt; 53 verts (Body), dist 0.2577; runner-up 81 at dist 0.2635))</t>
         </is>
       </c>
     </row>
@@ -4806,14 +4805,14 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C39" t="n">
         <v>0.9340000000000001</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Reviewed: coat sleeve, right, lower; the sleeve cuff (vertices mode), not a FINGER bone (101). Tool proposed 101. (1639 verts (A) -&gt; 53 verts (Body), dist 0.2577; runner-up 100 at dist 0.2635)</t>
+          <t>Reviewed (in game, the identity mod, 2026-09-25): the skin wears its coat as a MANTLE, its sleeves hanging empty behind the arms on a chain of their own; the whole chain onto his UPPER ARM (64 / 67). On his cuff piece and shoulder cloth the cuff jutted out at elbow height; on his clavicle the sleeves flared out at idle. (was: Reviewed: coat sleeve, right, lower; the sleeve cuff (vertices mode), not a FINGER bone (101). Tool proposed 101. (1639 verts (A) -&gt; 53 verts (Body), dist 0.2577; runner-up 100 at dist 0.2635))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hang Neuvillette's lower coat links from the skin's pelvis, not its knees
With the whole outfit on the main mesh (328ffab7) the rips were gone, but his lower coat links rode the
main mesh's knees and shins -- the nearest bones -- and cloth hanging 20-30 cm off a bending joint swung
with every bend of the idle pose: Neuvillette2's front panels splayed open over the lining,
Neuvillette3's cape folded inwards on the right, Kaiba's two cape halves crossed (Neuvillette5).
Groups 33, 34, 37-39, 41, 42, 45-47 now ride the pelvis (bone 0), so a hem hangs with the hips.

All ten mods checked front and turned round in game; other characters 1966 of 1966 files unchanged;
compiled == prototype on all ten. Draft workbook and Creating Remaps updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
+++ b/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
@@ -1093,14 +1093,14 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
         <v>0.964</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2631; runner-up 23 at dist 0.2112)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2631; runner-up 23 at dist 0.2112)</t>
         </is>
       </c>
     </row>
@@ -1109,14 +1109,14 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
         <v>0.5580000000000001</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 23 at dist 0.2687)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 23 at dist 0.2687)</t>
         </is>
       </c>
     </row>
@@ -1157,14 +1157,14 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
         <v>0.6889999999999999</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:9 at dist 0.2280)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:9 at dist 0.2280)</t>
         </is>
       </c>
     </row>
@@ -1173,14 +1173,14 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
         <v>0.294</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:21 at dist 0.3067)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:21 at dist 0.3067)</t>
         </is>
       </c>
     </row>
@@ -1189,14 +1189,14 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail (cyan trim); the skin coat's tail end, not the skin's CALF (cloth onto a leg). Tool proposed 6. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:24 at dist 0.3440))</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail (cyan trim); the skin coat's tail end, not the skin's CALF (cloth onto a leg). Tool proposed 6. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:24 at dist 0.3440))</t>
         </is>
       </c>
     </row>
@@ -1221,14 +1221,14 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
         <v>0.962</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2630; runner-up 43 at dist 0.2113)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 702 verts (Body) -&gt; 173 verts (Head), dist 0.2630; runner-up 43 at dist 0.2113)</t>
         </is>
       </c>
     </row>
@@ -1237,14 +1237,14 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
         <v>0.5580000000000001</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 43 at dist 0.2687)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 630 verts (Body) -&gt; 109 verts (A), dist 0.2263; runner-up 43 at dist 0.2687)</t>
         </is>
       </c>
     </row>
@@ -1285,14 +1285,14 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
         <v>0.6889999999999999</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:10 at dist 0.2280)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 225 verts (Body) -&gt; 109 verts (A), dist 0.2009; runner-up Coat:10 at dist 0.2280)</t>
         </is>
       </c>
     </row>
@@ -1301,14 +1301,14 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
         <v>0.373</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:22 at dist 0.3067)</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: 220 verts (Body) -&gt; 109 verts (A), dist 0.2176; runner-up Coat:22 at dist 0.3067)</t>
         </is>
       </c>
     </row>
@@ -1317,14 +1317,14 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F49" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on knees/shins, 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail, right; the skin coat's tail end, not the calf. Tool proposed 26. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:25 at dist 0.3440))</t>
+          <t>Reviewed (2026-09-25): whole outfit on the main mesh -- a cut between main mesh and Coat tore capes open in game (Neuvillette3/4/5); upper links on back-skirt bones, lower on the PELVIS (knees/shins swung the hem with the idle pose), 0/1 on the spine. | was: Reviewed (in game, Neuvillette3, 2026-09-24): his coat-tail chain goes WHOLE into the Coat, down its back panel by height -- split between the main mesh's back pieces and the Coat's tail ends, a vertex weighted to both was drawn by both components and the hem came out sawtoothed. (was: Reviewed: tip of the long back coat tail, right; the skin coat's tail end, not the calf. Tool proposed 26. (173 verts (Body) -&gt; 1106 verts (Body), dist 0.3287; runner-up Coat:25 at dist 0.3440))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Join The Council: 🧥🪡 The Coat Tailor, the 51st member
For the Neuvillette coat work: the seam, the pelvis links, the flap push and the mirrored lining.
The badges read 49 over a roster summing to 50 (two branches each bumped 48 -> 49); both count
SVGs now read 51, the roster's sum, and the ritual says to recompute before bumping. Credit row in
NeuvilletteRemapDraft.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
+++ b/Data/RemapDrafts/NeuvilletteRemapDraft.xlsx
@@ -63,17 +63,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -446,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="68" customWidth="1" min="1" max="1"/>
@@ -473,9 +476,17 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>🧥🪡 The Coat Tailor: The 51st member of The Council</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>